<commit_message>
Publish Belgrade_2017_WC, Pietermaritzburg_2017_MAR, Pitesti_2017_JWCH, Racice_2017_WCH, Szeged_2017_WC
</commit_message>
<xml_diff>
--- a/events/Pietermaritzburg_2017_MAR/Pietermaritzburg_2017_MAR_Results.xlsx
+++ b/events/Pietermaritzburg_2017_MAR/Pietermaritzburg_2017_MAR_Results.xlsx
@@ -4941,6 +4941,11 @@
           <t>01:35:13.250</t>
         </is>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>65695</t>
+        </is>
+      </c>
       <c r="S67" t="inlineStr">
         <is>
           <t>79147</t>
@@ -7970,6 +7975,11 @@
           <t>01:56:32.490</t>
         </is>
       </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>94098</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9946,6 +9956,11 @@
           <t>02:08:13.410</t>
         </is>
       </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -15994,6 +16009,11 @@
       <c r="R231" t="inlineStr">
         <is>
           <t>48405</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>94098</t>
         </is>
       </c>
     </row>
@@ -17130,7 +17150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D232"/>
+  <dimension ref="A1:D235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22237,6 +22257,72 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>65695</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Anne Hauge</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>SØRENSEN</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>94098</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Jean</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>VAN DER WESTHUIZEN</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Kristina</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>BEDEC</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>